<commit_message>
Support Excel product periods and existing exhibition append imports
</commit_message>
<xml_diff>
--- a/public/templates/LeiPort_Import_Template_v1.1.xlsx
+++ b/public/templates/LeiPort_Import_Template_v1.1.xlsx
@@ -94,12 +94,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
+    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -171,6 +172,12 @@
       <x:sz val="11"/>
       <x:color rgb="FF183B29"/>
       <x:name val="ＭＳ ゴシック"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF163F2B"/>
+      <x:name val="Yu Gothic"/>
     </x:font>
   </x:fonts>
   <x:fills count="9">
@@ -421,7 +428,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="71">
+  <x:cellXfs count="73">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -623,6 +630,10 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Normal" xfId="1"/>
@@ -643,8 +654,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LeiPortImportTable" displayName="LeiPortImportTable" ref="A3:O203">
-  <x:tableColumns count="15">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LeiPortImportTable" displayName="LeiPortImportTable" ref="A3:S203">
+  <x:tableColumns count="19">
     <x:tableColumn id="1" name="商品番号"/>
     <x:tableColumn id="2" name="商品名"/>
     <x:tableColumn id="3" name="カテゴリー"/>
@@ -660,6 +671,10 @@
     <x:tableColumn id="12" name="生産者"/>
     <x:tableColumn id="13" name="コメント"/>
     <x:tableColumn id="14" name="JFコード"/>
+    <x:tableColumn id="16" name="受付開始日"/>
+    <x:tableColumn id="17" name="受付終了日"/>
+    <x:tableColumn id="18" name="販売開始日"/>
+    <x:tableColumn id="19" name="販売終了日"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -955,7 +970,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="14.25"/>
   <x:cols>
     <x:col min="1" max="1" width="11" customWidth="1"/>
@@ -972,6 +987,10 @@
     <x:col min="13" max="13" width="18" customWidth="1"/>
     <x:col min="14" max="14" width="34" customWidth="1"/>
     <x:col min="15" max="15" width="14" customWidth="1"/>
+    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1058,6 +1077,18 @@
       <x:c r="O3" s="20" t="str">
         <x:v>JFコード</x:v>
       </x:c>
+      <x:c r="P3" s="71" t="str">
+        <x:v>受付開始日</x:v>
+      </x:c>
+      <x:c r="Q3" s="71" t="str">
+        <x:v>受付終了日</x:v>
+      </x:c>
+      <x:c r="R3" s="71" t="str">
+        <x:v>販売開始日</x:v>
+      </x:c>
+      <x:c r="S3" s="71" t="str">
+        <x:v>販売終了日</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="28.5">
       <x:c r="A4" s="21">
@@ -1103,6 +1134,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="O4" s="25"/>
+      <x:c r="P4" s="72"/>
+      <x:c r="Q4" s="72"/>
+      <x:c r="R4" s="72"/>
+      <x:c r="S4" s="72"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="21"/>
@@ -1120,6 +1155,10 @@
       <x:c r="M5" s="26"/>
       <x:c r="N5" s="26"/>
       <x:c r="O5" s="27"/>
+      <x:c r="P5" s="72"/>
+      <x:c r="Q5" s="72"/>
+      <x:c r="R5" s="72"/>
+      <x:c r="S5" s="72"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="21"/>
@@ -1137,6 +1176,10 @@
       <x:c r="M6" s="26"/>
       <x:c r="N6" s="26"/>
       <x:c r="O6" s="27"/>
+      <x:c r="P6" s="72"/>
+      <x:c r="Q6" s="72"/>
+      <x:c r="R6" s="72"/>
+      <x:c r="S6" s="72"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="21"/>
@@ -1154,6 +1197,10 @@
       <x:c r="M7" s="26"/>
       <x:c r="N7" s="26"/>
       <x:c r="O7" s="27"/>
+      <x:c r="P7" s="72"/>
+      <x:c r="Q7" s="72"/>
+      <x:c r="R7" s="72"/>
+      <x:c r="S7" s="72"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="21"/>
@@ -1171,6 +1218,10 @@
       <x:c r="M8" s="26"/>
       <x:c r="N8" s="26"/>
       <x:c r="O8" s="27"/>
+      <x:c r="P8" s="72"/>
+      <x:c r="Q8" s="72"/>
+      <x:c r="R8" s="72"/>
+      <x:c r="S8" s="72"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="21"/>
@@ -1188,6 +1239,10 @@
       <x:c r="M9" s="26"/>
       <x:c r="N9" s="26"/>
       <x:c r="O9" s="27"/>
+      <x:c r="P9" s="72"/>
+      <x:c r="Q9" s="72"/>
+      <x:c r="R9" s="72"/>
+      <x:c r="S9" s="72"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="21"/>
@@ -1205,6 +1260,10 @@
       <x:c r="M10" s="26"/>
       <x:c r="N10" s="26"/>
       <x:c r="O10" s="27"/>
+      <x:c r="P10" s="72"/>
+      <x:c r="Q10" s="72"/>
+      <x:c r="R10" s="72"/>
+      <x:c r="S10" s="72"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="21"/>
@@ -1222,6 +1281,10 @@
       <x:c r="M11" s="26"/>
       <x:c r="N11" s="26"/>
       <x:c r="O11" s="27"/>
+      <x:c r="P11" s="72"/>
+      <x:c r="Q11" s="72"/>
+      <x:c r="R11" s="72"/>
+      <x:c r="S11" s="72"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="21"/>
@@ -1239,6 +1302,10 @@
       <x:c r="M12" s="26"/>
       <x:c r="N12" s="26"/>
       <x:c r="O12" s="27"/>
+      <x:c r="P12" s="72"/>
+      <x:c r="Q12" s="72"/>
+      <x:c r="R12" s="72"/>
+      <x:c r="S12" s="72"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="21"/>
@@ -1256,6 +1323,10 @@
       <x:c r="M13" s="26"/>
       <x:c r="N13" s="26"/>
       <x:c r="O13" s="27"/>
+      <x:c r="P13" s="72"/>
+      <x:c r="Q13" s="72"/>
+      <x:c r="R13" s="72"/>
+      <x:c r="S13" s="72"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="21"/>
@@ -1273,6 +1344,10 @@
       <x:c r="M14" s="26"/>
       <x:c r="N14" s="26"/>
       <x:c r="O14" s="27"/>
+      <x:c r="P14" s="72"/>
+      <x:c r="Q14" s="72"/>
+      <x:c r="R14" s="72"/>
+      <x:c r="S14" s="72"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="21"/>
@@ -1290,6 +1365,10 @@
       <x:c r="M15" s="26"/>
       <x:c r="N15" s="26"/>
       <x:c r="O15" s="27"/>
+      <x:c r="P15" s="72"/>
+      <x:c r="Q15" s="72"/>
+      <x:c r="R15" s="72"/>
+      <x:c r="S15" s="72"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="21"/>
@@ -1307,6 +1386,10 @@
       <x:c r="M16" s="26"/>
       <x:c r="N16" s="26"/>
       <x:c r="O16" s="27"/>
+      <x:c r="P16" s="72"/>
+      <x:c r="Q16" s="72"/>
+      <x:c r="R16" s="72"/>
+      <x:c r="S16" s="72"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="21"/>
@@ -1324,6 +1407,10 @@
       <x:c r="M17" s="26"/>
       <x:c r="N17" s="26"/>
       <x:c r="O17" s="27"/>
+      <x:c r="P17" s="72"/>
+      <x:c r="Q17" s="72"/>
+      <x:c r="R17" s="72"/>
+      <x:c r="S17" s="72"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="21"/>
@@ -1341,6 +1428,10 @@
       <x:c r="M18" s="26"/>
       <x:c r="N18" s="26"/>
       <x:c r="O18" s="27"/>
+      <x:c r="P18" s="72"/>
+      <x:c r="Q18" s="72"/>
+      <x:c r="R18" s="72"/>
+      <x:c r="S18" s="72"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="21"/>
@@ -1358,6 +1449,10 @@
       <x:c r="M19" s="26"/>
       <x:c r="N19" s="26"/>
       <x:c r="O19" s="27"/>
+      <x:c r="P19" s="72"/>
+      <x:c r="Q19" s="72"/>
+      <x:c r="R19" s="72"/>
+      <x:c r="S19" s="72"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="21"/>
@@ -1375,6 +1470,10 @@
       <x:c r="M20" s="26"/>
       <x:c r="N20" s="26"/>
       <x:c r="O20" s="27"/>
+      <x:c r="P20" s="72"/>
+      <x:c r="Q20" s="72"/>
+      <x:c r="R20" s="72"/>
+      <x:c r="S20" s="72"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="21"/>
@@ -1392,6 +1491,10 @@
       <x:c r="M21" s="26"/>
       <x:c r="N21" s="26"/>
       <x:c r="O21" s="27"/>
+      <x:c r="P21" s="72"/>
+      <x:c r="Q21" s="72"/>
+      <x:c r="R21" s="72"/>
+      <x:c r="S21" s="72"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="21"/>
@@ -1409,6 +1512,10 @@
       <x:c r="M22" s="26"/>
       <x:c r="N22" s="26"/>
       <x:c r="O22" s="27"/>
+      <x:c r="P22" s="72"/>
+      <x:c r="Q22" s="72"/>
+      <x:c r="R22" s="72"/>
+      <x:c r="S22" s="72"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="21"/>
@@ -1426,6 +1533,10 @@
       <x:c r="M23" s="26"/>
       <x:c r="N23" s="26"/>
       <x:c r="O23" s="27"/>
+      <x:c r="P23" s="72"/>
+      <x:c r="Q23" s="72"/>
+      <x:c r="R23" s="72"/>
+      <x:c r="S23" s="72"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="21"/>
@@ -1443,6 +1554,10 @@
       <x:c r="M24" s="26"/>
       <x:c r="N24" s="26"/>
       <x:c r="O24" s="27"/>
+      <x:c r="P24" s="72"/>
+      <x:c r="Q24" s="72"/>
+      <x:c r="R24" s="72"/>
+      <x:c r="S24" s="72"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="21"/>
@@ -1460,6 +1575,10 @@
       <x:c r="M25" s="26"/>
       <x:c r="N25" s="26"/>
       <x:c r="O25" s="27"/>
+      <x:c r="P25" s="72"/>
+      <x:c r="Q25" s="72"/>
+      <x:c r="R25" s="72"/>
+      <x:c r="S25" s="72"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="21"/>
@@ -1477,6 +1596,10 @@
       <x:c r="M26" s="26"/>
       <x:c r="N26" s="26"/>
       <x:c r="O26" s="27"/>
+      <x:c r="P26" s="72"/>
+      <x:c r="Q26" s="72"/>
+      <x:c r="R26" s="72"/>
+      <x:c r="S26" s="72"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="21"/>
@@ -1494,6 +1617,10 @@
       <x:c r="M27" s="26"/>
       <x:c r="N27" s="26"/>
       <x:c r="O27" s="27"/>
+      <x:c r="P27" s="72"/>
+      <x:c r="Q27" s="72"/>
+      <x:c r="R27" s="72"/>
+      <x:c r="S27" s="72"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="21"/>
@@ -1511,6 +1638,10 @@
       <x:c r="M28" s="26"/>
       <x:c r="N28" s="26"/>
       <x:c r="O28" s="27"/>
+      <x:c r="P28" s="72"/>
+      <x:c r="Q28" s="72"/>
+      <x:c r="R28" s="72"/>
+      <x:c r="S28" s="72"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="21"/>
@@ -1528,6 +1659,10 @@
       <x:c r="M29" s="26"/>
       <x:c r="N29" s="26"/>
       <x:c r="O29" s="27"/>
+      <x:c r="P29" s="72"/>
+      <x:c r="Q29" s="72"/>
+      <x:c r="R29" s="72"/>
+      <x:c r="S29" s="72"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="21"/>
@@ -1545,6 +1680,10 @@
       <x:c r="M30" s="26"/>
       <x:c r="N30" s="26"/>
       <x:c r="O30" s="27"/>
+      <x:c r="P30" s="72"/>
+      <x:c r="Q30" s="72"/>
+      <x:c r="R30" s="72"/>
+      <x:c r="S30" s="72"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="21"/>
@@ -1562,6 +1701,10 @@
       <x:c r="M31" s="26"/>
       <x:c r="N31" s="26"/>
       <x:c r="O31" s="27"/>
+      <x:c r="P31" s="72"/>
+      <x:c r="Q31" s="72"/>
+      <x:c r="R31" s="72"/>
+      <x:c r="S31" s="72"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="21"/>
@@ -1579,6 +1722,10 @@
       <x:c r="M32" s="26"/>
       <x:c r="N32" s="26"/>
       <x:c r="O32" s="27"/>
+      <x:c r="P32" s="72"/>
+      <x:c r="Q32" s="72"/>
+      <x:c r="R32" s="72"/>
+      <x:c r="S32" s="72"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="21"/>
@@ -1596,6 +1743,10 @@
       <x:c r="M33" s="26"/>
       <x:c r="N33" s="26"/>
       <x:c r="O33" s="27"/>
+      <x:c r="P33" s="72"/>
+      <x:c r="Q33" s="72"/>
+      <x:c r="R33" s="72"/>
+      <x:c r="S33" s="72"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="21"/>
@@ -1613,6 +1764,10 @@
       <x:c r="M34" s="26"/>
       <x:c r="N34" s="26"/>
       <x:c r="O34" s="27"/>
+      <x:c r="P34" s="72"/>
+      <x:c r="Q34" s="72"/>
+      <x:c r="R34" s="72"/>
+      <x:c r="S34" s="72"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="21"/>
@@ -1630,6 +1785,10 @@
       <x:c r="M35" s="26"/>
       <x:c r="N35" s="26"/>
       <x:c r="O35" s="27"/>
+      <x:c r="P35" s="72"/>
+      <x:c r="Q35" s="72"/>
+      <x:c r="R35" s="72"/>
+      <x:c r="S35" s="72"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="21"/>
@@ -1647,6 +1806,10 @@
       <x:c r="M36" s="26"/>
       <x:c r="N36" s="26"/>
       <x:c r="O36" s="27"/>
+      <x:c r="P36" s="72"/>
+      <x:c r="Q36" s="72"/>
+      <x:c r="R36" s="72"/>
+      <x:c r="S36" s="72"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="21"/>
@@ -1664,6 +1827,10 @@
       <x:c r="M37" s="26"/>
       <x:c r="N37" s="26"/>
       <x:c r="O37" s="27"/>
+      <x:c r="P37" s="72"/>
+      <x:c r="Q37" s="72"/>
+      <x:c r="R37" s="72"/>
+      <x:c r="S37" s="72"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="21"/>
@@ -1681,6 +1848,10 @@
       <x:c r="M38" s="26"/>
       <x:c r="N38" s="26"/>
       <x:c r="O38" s="27"/>
+      <x:c r="P38" s="72"/>
+      <x:c r="Q38" s="72"/>
+      <x:c r="R38" s="72"/>
+      <x:c r="S38" s="72"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="21"/>
@@ -1698,6 +1869,10 @@
       <x:c r="M39" s="26"/>
       <x:c r="N39" s="26"/>
       <x:c r="O39" s="27"/>
+      <x:c r="P39" s="72"/>
+      <x:c r="Q39" s="72"/>
+      <x:c r="R39" s="72"/>
+      <x:c r="S39" s="72"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="21"/>
@@ -1715,6 +1890,10 @@
       <x:c r="M40" s="26"/>
       <x:c r="N40" s="26"/>
       <x:c r="O40" s="27"/>
+      <x:c r="P40" s="72"/>
+      <x:c r="Q40" s="72"/>
+      <x:c r="R40" s="72"/>
+      <x:c r="S40" s="72"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="21"/>
@@ -1732,6 +1911,10 @@
       <x:c r="M41" s="26"/>
       <x:c r="N41" s="26"/>
       <x:c r="O41" s="27"/>
+      <x:c r="P41" s="72"/>
+      <x:c r="Q41" s="72"/>
+      <x:c r="R41" s="72"/>
+      <x:c r="S41" s="72"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="21"/>
@@ -1749,6 +1932,10 @@
       <x:c r="M42" s="26"/>
       <x:c r="N42" s="26"/>
       <x:c r="O42" s="27"/>
+      <x:c r="P42" s="72"/>
+      <x:c r="Q42" s="72"/>
+      <x:c r="R42" s="72"/>
+      <x:c r="S42" s="72"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="21"/>
@@ -1766,6 +1953,10 @@
       <x:c r="M43" s="26"/>
       <x:c r="N43" s="26"/>
       <x:c r="O43" s="27"/>
+      <x:c r="P43" s="72"/>
+      <x:c r="Q43" s="72"/>
+      <x:c r="R43" s="72"/>
+      <x:c r="S43" s="72"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="21"/>
@@ -1783,6 +1974,10 @@
       <x:c r="M44" s="26"/>
       <x:c r="N44" s="26"/>
       <x:c r="O44" s="27"/>
+      <x:c r="P44" s="72"/>
+      <x:c r="Q44" s="72"/>
+      <x:c r="R44" s="72"/>
+      <x:c r="S44" s="72"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="21"/>
@@ -1800,6 +1995,10 @@
       <x:c r="M45" s="26"/>
       <x:c r="N45" s="26"/>
       <x:c r="O45" s="27"/>
+      <x:c r="P45" s="72"/>
+      <x:c r="Q45" s="72"/>
+      <x:c r="R45" s="72"/>
+      <x:c r="S45" s="72"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="21"/>
@@ -1817,6 +2016,10 @@
       <x:c r="M46" s="26"/>
       <x:c r="N46" s="26"/>
       <x:c r="O46" s="27"/>
+      <x:c r="P46" s="72"/>
+      <x:c r="Q46" s="72"/>
+      <x:c r="R46" s="72"/>
+      <x:c r="S46" s="72"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="21"/>
@@ -1834,6 +2037,10 @@
       <x:c r="M47" s="26"/>
       <x:c r="N47" s="26"/>
       <x:c r="O47" s="27"/>
+      <x:c r="P47" s="72"/>
+      <x:c r="Q47" s="72"/>
+      <x:c r="R47" s="72"/>
+      <x:c r="S47" s="72"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="21"/>
@@ -1851,6 +2058,10 @@
       <x:c r="M48" s="26"/>
       <x:c r="N48" s="26"/>
       <x:c r="O48" s="27"/>
+      <x:c r="P48" s="72"/>
+      <x:c r="Q48" s="72"/>
+      <x:c r="R48" s="72"/>
+      <x:c r="S48" s="72"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="21"/>
@@ -1868,6 +2079,10 @@
       <x:c r="M49" s="26"/>
       <x:c r="N49" s="26"/>
       <x:c r="O49" s="27"/>
+      <x:c r="P49" s="72"/>
+      <x:c r="Q49" s="72"/>
+      <x:c r="R49" s="72"/>
+      <x:c r="S49" s="72"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="21"/>
@@ -1885,6 +2100,10 @@
       <x:c r="M50" s="26"/>
       <x:c r="N50" s="26"/>
       <x:c r="O50" s="27"/>
+      <x:c r="P50" s="72"/>
+      <x:c r="Q50" s="72"/>
+      <x:c r="R50" s="72"/>
+      <x:c r="S50" s="72"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="21"/>
@@ -1902,6 +2121,10 @@
       <x:c r="M51" s="26"/>
       <x:c r="N51" s="26"/>
       <x:c r="O51" s="27"/>
+      <x:c r="P51" s="72"/>
+      <x:c r="Q51" s="72"/>
+      <x:c r="R51" s="72"/>
+      <x:c r="S51" s="72"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="21"/>
@@ -1919,6 +2142,10 @@
       <x:c r="M52" s="26"/>
       <x:c r="N52" s="26"/>
       <x:c r="O52" s="27"/>
+      <x:c r="P52" s="72"/>
+      <x:c r="Q52" s="72"/>
+      <x:c r="R52" s="72"/>
+      <x:c r="S52" s="72"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="21"/>
@@ -1936,6 +2163,10 @@
       <x:c r="M53" s="26"/>
       <x:c r="N53" s="26"/>
       <x:c r="O53" s="27"/>
+      <x:c r="P53" s="72"/>
+      <x:c r="Q53" s="72"/>
+      <x:c r="R53" s="72"/>
+      <x:c r="S53" s="72"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="21"/>
@@ -1953,6 +2184,10 @@
       <x:c r="M54" s="26"/>
       <x:c r="N54" s="26"/>
       <x:c r="O54" s="27"/>
+      <x:c r="P54" s="72"/>
+      <x:c r="Q54" s="72"/>
+      <x:c r="R54" s="72"/>
+      <x:c r="S54" s="72"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="21"/>
@@ -1970,6 +2205,10 @@
       <x:c r="M55" s="26"/>
       <x:c r="N55" s="26"/>
       <x:c r="O55" s="27"/>
+      <x:c r="P55" s="72"/>
+      <x:c r="Q55" s="72"/>
+      <x:c r="R55" s="72"/>
+      <x:c r="S55" s="72"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="21"/>
@@ -1987,6 +2226,10 @@
       <x:c r="M56" s="26"/>
       <x:c r="N56" s="26"/>
       <x:c r="O56" s="27"/>
+      <x:c r="P56" s="72"/>
+      <x:c r="Q56" s="72"/>
+      <x:c r="R56" s="72"/>
+      <x:c r="S56" s="72"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="21"/>
@@ -2004,6 +2247,10 @@
       <x:c r="M57" s="26"/>
       <x:c r="N57" s="26"/>
       <x:c r="O57" s="27"/>
+      <x:c r="P57" s="72"/>
+      <x:c r="Q57" s="72"/>
+      <x:c r="R57" s="72"/>
+      <x:c r="S57" s="72"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="21"/>
@@ -2021,6 +2268,10 @@
       <x:c r="M58" s="26"/>
       <x:c r="N58" s="26"/>
       <x:c r="O58" s="27"/>
+      <x:c r="P58" s="72"/>
+      <x:c r="Q58" s="72"/>
+      <x:c r="R58" s="72"/>
+      <x:c r="S58" s="72"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="21"/>
@@ -2038,6 +2289,10 @@
       <x:c r="M59" s="26"/>
       <x:c r="N59" s="26"/>
       <x:c r="O59" s="27"/>
+      <x:c r="P59" s="72"/>
+      <x:c r="Q59" s="72"/>
+      <x:c r="R59" s="72"/>
+      <x:c r="S59" s="72"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="21"/>
@@ -2055,6 +2310,10 @@
       <x:c r="M60" s="26"/>
       <x:c r="N60" s="26"/>
       <x:c r="O60" s="27"/>
+      <x:c r="P60" s="72"/>
+      <x:c r="Q60" s="72"/>
+      <x:c r="R60" s="72"/>
+      <x:c r="S60" s="72"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="21"/>
@@ -2072,6 +2331,10 @@
       <x:c r="M61" s="26"/>
       <x:c r="N61" s="26"/>
       <x:c r="O61" s="27"/>
+      <x:c r="P61" s="72"/>
+      <x:c r="Q61" s="72"/>
+      <x:c r="R61" s="72"/>
+      <x:c r="S61" s="72"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="21"/>
@@ -2089,6 +2352,10 @@
       <x:c r="M62" s="26"/>
       <x:c r="N62" s="26"/>
       <x:c r="O62" s="27"/>
+      <x:c r="P62" s="72"/>
+      <x:c r="Q62" s="72"/>
+      <x:c r="R62" s="72"/>
+      <x:c r="S62" s="72"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="21"/>
@@ -2106,6 +2373,10 @@
       <x:c r="M63" s="26"/>
       <x:c r="N63" s="26"/>
       <x:c r="O63" s="27"/>
+      <x:c r="P63" s="72"/>
+      <x:c r="Q63" s="72"/>
+      <x:c r="R63" s="72"/>
+      <x:c r="S63" s="72"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="21"/>
@@ -2123,6 +2394,10 @@
       <x:c r="M64" s="26"/>
       <x:c r="N64" s="26"/>
       <x:c r="O64" s="27"/>
+      <x:c r="P64" s="72"/>
+      <x:c r="Q64" s="72"/>
+      <x:c r="R64" s="72"/>
+      <x:c r="S64" s="72"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="21"/>
@@ -2140,6 +2415,10 @@
       <x:c r="M65" s="26"/>
       <x:c r="N65" s="26"/>
       <x:c r="O65" s="27"/>
+      <x:c r="P65" s="72"/>
+      <x:c r="Q65" s="72"/>
+      <x:c r="R65" s="72"/>
+      <x:c r="S65" s="72"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="21"/>
@@ -2157,6 +2436,10 @@
       <x:c r="M66" s="26"/>
       <x:c r="N66" s="26"/>
       <x:c r="O66" s="27"/>
+      <x:c r="P66" s="72"/>
+      <x:c r="Q66" s="72"/>
+      <x:c r="R66" s="72"/>
+      <x:c r="S66" s="72"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="21"/>
@@ -2174,6 +2457,10 @@
       <x:c r="M67" s="26"/>
       <x:c r="N67" s="26"/>
       <x:c r="O67" s="27"/>
+      <x:c r="P67" s="72"/>
+      <x:c r="Q67" s="72"/>
+      <x:c r="R67" s="72"/>
+      <x:c r="S67" s="72"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="21"/>
@@ -2191,6 +2478,10 @@
       <x:c r="M68" s="26"/>
       <x:c r="N68" s="26"/>
       <x:c r="O68" s="27"/>
+      <x:c r="P68" s="72"/>
+      <x:c r="Q68" s="72"/>
+      <x:c r="R68" s="72"/>
+      <x:c r="S68" s="72"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="21"/>
@@ -2208,6 +2499,10 @@
       <x:c r="M69" s="26"/>
       <x:c r="N69" s="26"/>
       <x:c r="O69" s="27"/>
+      <x:c r="P69" s="72"/>
+      <x:c r="Q69" s="72"/>
+      <x:c r="R69" s="72"/>
+      <x:c r="S69" s="72"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="21"/>
@@ -2225,6 +2520,10 @@
       <x:c r="M70" s="26"/>
       <x:c r="N70" s="26"/>
       <x:c r="O70" s="27"/>
+      <x:c r="P70" s="72"/>
+      <x:c r="Q70" s="72"/>
+      <x:c r="R70" s="72"/>
+      <x:c r="S70" s="72"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="21"/>
@@ -2242,6 +2541,10 @@
       <x:c r="M71" s="26"/>
       <x:c r="N71" s="26"/>
       <x:c r="O71" s="27"/>
+      <x:c r="P71" s="72"/>
+      <x:c r="Q71" s="72"/>
+      <x:c r="R71" s="72"/>
+      <x:c r="S71" s="72"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="21"/>
@@ -2259,6 +2562,10 @@
       <x:c r="M72" s="26"/>
       <x:c r="N72" s="26"/>
       <x:c r="O72" s="27"/>
+      <x:c r="P72" s="72"/>
+      <x:c r="Q72" s="72"/>
+      <x:c r="R72" s="72"/>
+      <x:c r="S72" s="72"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="21"/>
@@ -2276,6 +2583,10 @@
       <x:c r="M73" s="26"/>
       <x:c r="N73" s="26"/>
       <x:c r="O73" s="27"/>
+      <x:c r="P73" s="72"/>
+      <x:c r="Q73" s="72"/>
+      <x:c r="R73" s="72"/>
+      <x:c r="S73" s="72"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="21"/>
@@ -2293,6 +2604,10 @@
       <x:c r="M74" s="26"/>
       <x:c r="N74" s="26"/>
       <x:c r="O74" s="27"/>
+      <x:c r="P74" s="72"/>
+      <x:c r="Q74" s="72"/>
+      <x:c r="R74" s="72"/>
+      <x:c r="S74" s="72"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="21"/>
@@ -2310,6 +2625,10 @@
       <x:c r="M75" s="26"/>
       <x:c r="N75" s="26"/>
       <x:c r="O75" s="27"/>
+      <x:c r="P75" s="72"/>
+      <x:c r="Q75" s="72"/>
+      <x:c r="R75" s="72"/>
+      <x:c r="S75" s="72"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="21"/>
@@ -2327,6 +2646,10 @@
       <x:c r="M76" s="26"/>
       <x:c r="N76" s="26"/>
       <x:c r="O76" s="27"/>
+      <x:c r="P76" s="72"/>
+      <x:c r="Q76" s="72"/>
+      <x:c r="R76" s="72"/>
+      <x:c r="S76" s="72"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="21"/>
@@ -2344,6 +2667,10 @@
       <x:c r="M77" s="26"/>
       <x:c r="N77" s="26"/>
       <x:c r="O77" s="27"/>
+      <x:c r="P77" s="72"/>
+      <x:c r="Q77" s="72"/>
+      <x:c r="R77" s="72"/>
+      <x:c r="S77" s="72"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="21"/>
@@ -2361,6 +2688,10 @@
       <x:c r="M78" s="26"/>
       <x:c r="N78" s="26"/>
       <x:c r="O78" s="27"/>
+      <x:c r="P78" s="72"/>
+      <x:c r="Q78" s="72"/>
+      <x:c r="R78" s="72"/>
+      <x:c r="S78" s="72"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="21"/>
@@ -2378,6 +2709,10 @@
       <x:c r="M79" s="26"/>
       <x:c r="N79" s="26"/>
       <x:c r="O79" s="27"/>
+      <x:c r="P79" s="72"/>
+      <x:c r="Q79" s="72"/>
+      <x:c r="R79" s="72"/>
+      <x:c r="S79" s="72"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="21"/>
@@ -2395,6 +2730,10 @@
       <x:c r="M80" s="26"/>
       <x:c r="N80" s="26"/>
       <x:c r="O80" s="27"/>
+      <x:c r="P80" s="72"/>
+      <x:c r="Q80" s="72"/>
+      <x:c r="R80" s="72"/>
+      <x:c r="S80" s="72"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="21"/>
@@ -2412,6 +2751,10 @@
       <x:c r="M81" s="26"/>
       <x:c r="N81" s="26"/>
       <x:c r="O81" s="27"/>
+      <x:c r="P81" s="72"/>
+      <x:c r="Q81" s="72"/>
+      <x:c r="R81" s="72"/>
+      <x:c r="S81" s="72"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="21"/>
@@ -2429,6 +2772,10 @@
       <x:c r="M82" s="26"/>
       <x:c r="N82" s="26"/>
       <x:c r="O82" s="27"/>
+      <x:c r="P82" s="72"/>
+      <x:c r="Q82" s="72"/>
+      <x:c r="R82" s="72"/>
+      <x:c r="S82" s="72"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="21"/>
@@ -2446,6 +2793,10 @@
       <x:c r="M83" s="26"/>
       <x:c r="N83" s="26"/>
       <x:c r="O83" s="27"/>
+      <x:c r="P83" s="72"/>
+      <x:c r="Q83" s="72"/>
+      <x:c r="R83" s="72"/>
+      <x:c r="S83" s="72"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="21"/>
@@ -2463,6 +2814,10 @@
       <x:c r="M84" s="26"/>
       <x:c r="N84" s="26"/>
       <x:c r="O84" s="27"/>
+      <x:c r="P84" s="72"/>
+      <x:c r="Q84" s="72"/>
+      <x:c r="R84" s="72"/>
+      <x:c r="S84" s="72"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="21"/>
@@ -2480,6 +2835,10 @@
       <x:c r="M85" s="26"/>
       <x:c r="N85" s="26"/>
       <x:c r="O85" s="27"/>
+      <x:c r="P85" s="72"/>
+      <x:c r="Q85" s="72"/>
+      <x:c r="R85" s="72"/>
+      <x:c r="S85" s="72"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="21"/>
@@ -2497,6 +2856,10 @@
       <x:c r="M86" s="26"/>
       <x:c r="N86" s="26"/>
       <x:c r="O86" s="27"/>
+      <x:c r="P86" s="72"/>
+      <x:c r="Q86" s="72"/>
+      <x:c r="R86" s="72"/>
+      <x:c r="S86" s="72"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="21"/>
@@ -2514,6 +2877,10 @@
       <x:c r="M87" s="26"/>
       <x:c r="N87" s="26"/>
       <x:c r="O87" s="27"/>
+      <x:c r="P87" s="72"/>
+      <x:c r="Q87" s="72"/>
+      <x:c r="R87" s="72"/>
+      <x:c r="S87" s="72"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="21"/>
@@ -2531,6 +2898,10 @@
       <x:c r="M88" s="26"/>
       <x:c r="N88" s="26"/>
       <x:c r="O88" s="27"/>
+      <x:c r="P88" s="72"/>
+      <x:c r="Q88" s="72"/>
+      <x:c r="R88" s="72"/>
+      <x:c r="S88" s="72"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="21"/>
@@ -2548,6 +2919,10 @@
       <x:c r="M89" s="26"/>
       <x:c r="N89" s="26"/>
       <x:c r="O89" s="27"/>
+      <x:c r="P89" s="72"/>
+      <x:c r="Q89" s="72"/>
+      <x:c r="R89" s="72"/>
+      <x:c r="S89" s="72"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="21"/>
@@ -2565,6 +2940,10 @@
       <x:c r="M90" s="26"/>
       <x:c r="N90" s="26"/>
       <x:c r="O90" s="27"/>
+      <x:c r="P90" s="72"/>
+      <x:c r="Q90" s="72"/>
+      <x:c r="R90" s="72"/>
+      <x:c r="S90" s="72"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="21"/>
@@ -2582,6 +2961,10 @@
       <x:c r="M91" s="26"/>
       <x:c r="N91" s="26"/>
       <x:c r="O91" s="27"/>
+      <x:c r="P91" s="72"/>
+      <x:c r="Q91" s="72"/>
+      <x:c r="R91" s="72"/>
+      <x:c r="S91" s="72"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="21"/>
@@ -2599,6 +2982,10 @@
       <x:c r="M92" s="26"/>
       <x:c r="N92" s="26"/>
       <x:c r="O92" s="27"/>
+      <x:c r="P92" s="72"/>
+      <x:c r="Q92" s="72"/>
+      <x:c r="R92" s="72"/>
+      <x:c r="S92" s="72"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="21"/>
@@ -2616,6 +3003,10 @@
       <x:c r="M93" s="26"/>
       <x:c r="N93" s="26"/>
       <x:c r="O93" s="27"/>
+      <x:c r="P93" s="72"/>
+      <x:c r="Q93" s="72"/>
+      <x:c r="R93" s="72"/>
+      <x:c r="S93" s="72"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="21"/>
@@ -2633,6 +3024,10 @@
       <x:c r="M94" s="26"/>
       <x:c r="N94" s="26"/>
       <x:c r="O94" s="27"/>
+      <x:c r="P94" s="72"/>
+      <x:c r="Q94" s="72"/>
+      <x:c r="R94" s="72"/>
+      <x:c r="S94" s="72"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="21"/>
@@ -2650,6 +3045,10 @@
       <x:c r="M95" s="26"/>
       <x:c r="N95" s="26"/>
       <x:c r="O95" s="27"/>
+      <x:c r="P95" s="72"/>
+      <x:c r="Q95" s="72"/>
+      <x:c r="R95" s="72"/>
+      <x:c r="S95" s="72"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="21"/>
@@ -2667,6 +3066,10 @@
       <x:c r="M96" s="26"/>
       <x:c r="N96" s="26"/>
       <x:c r="O96" s="27"/>
+      <x:c r="P96" s="72"/>
+      <x:c r="Q96" s="72"/>
+      <x:c r="R96" s="72"/>
+      <x:c r="S96" s="72"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="21"/>
@@ -2684,6 +3087,10 @@
       <x:c r="M97" s="26"/>
       <x:c r="N97" s="26"/>
       <x:c r="O97" s="27"/>
+      <x:c r="P97" s="72"/>
+      <x:c r="Q97" s="72"/>
+      <x:c r="R97" s="72"/>
+      <x:c r="S97" s="72"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="21"/>
@@ -2701,6 +3108,10 @@
       <x:c r="M98" s="26"/>
       <x:c r="N98" s="26"/>
       <x:c r="O98" s="27"/>
+      <x:c r="P98" s="72"/>
+      <x:c r="Q98" s="72"/>
+      <x:c r="R98" s="72"/>
+      <x:c r="S98" s="72"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="21"/>
@@ -2718,6 +3129,10 @@
       <x:c r="M99" s="26"/>
       <x:c r="N99" s="26"/>
       <x:c r="O99" s="27"/>
+      <x:c r="P99" s="72"/>
+      <x:c r="Q99" s="72"/>
+      <x:c r="R99" s="72"/>
+      <x:c r="S99" s="72"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="21"/>
@@ -2735,6 +3150,10 @@
       <x:c r="M100" s="26"/>
       <x:c r="N100" s="26"/>
       <x:c r="O100" s="27"/>
+      <x:c r="P100" s="72"/>
+      <x:c r="Q100" s="72"/>
+      <x:c r="R100" s="72"/>
+      <x:c r="S100" s="72"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="21"/>
@@ -2752,6 +3171,10 @@
       <x:c r="M101" s="26"/>
       <x:c r="N101" s="26"/>
       <x:c r="O101" s="27"/>
+      <x:c r="P101" s="72"/>
+      <x:c r="Q101" s="72"/>
+      <x:c r="R101" s="72"/>
+      <x:c r="S101" s="72"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="21"/>
@@ -2769,6 +3192,10 @@
       <x:c r="M102" s="26"/>
       <x:c r="N102" s="26"/>
       <x:c r="O102" s="27"/>
+      <x:c r="P102" s="72"/>
+      <x:c r="Q102" s="72"/>
+      <x:c r="R102" s="72"/>
+      <x:c r="S102" s="72"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="21"/>
@@ -2786,6 +3213,10 @@
       <x:c r="M103" s="26"/>
       <x:c r="N103" s="26"/>
       <x:c r="O103" s="27"/>
+      <x:c r="P103" s="72"/>
+      <x:c r="Q103" s="72"/>
+      <x:c r="R103" s="72"/>
+      <x:c r="S103" s="72"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="21"/>
@@ -2803,6 +3234,10 @@
       <x:c r="M104" s="26"/>
       <x:c r="N104" s="26"/>
       <x:c r="O104" s="27"/>
+      <x:c r="P104" s="72"/>
+      <x:c r="Q104" s="72"/>
+      <x:c r="R104" s="72"/>
+      <x:c r="S104" s="72"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="21"/>
@@ -2820,6 +3255,10 @@
       <x:c r="M105" s="26"/>
       <x:c r="N105" s="26"/>
       <x:c r="O105" s="27"/>
+      <x:c r="P105" s="72"/>
+      <x:c r="Q105" s="72"/>
+      <x:c r="R105" s="72"/>
+      <x:c r="S105" s="72"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="21"/>
@@ -2837,6 +3276,10 @@
       <x:c r="M106" s="26"/>
       <x:c r="N106" s="26"/>
       <x:c r="O106" s="27"/>
+      <x:c r="P106" s="72"/>
+      <x:c r="Q106" s="72"/>
+      <x:c r="R106" s="72"/>
+      <x:c r="S106" s="72"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="21"/>
@@ -2854,6 +3297,10 @@
       <x:c r="M107" s="26"/>
       <x:c r="N107" s="26"/>
       <x:c r="O107" s="27"/>
+      <x:c r="P107" s="72"/>
+      <x:c r="Q107" s="72"/>
+      <x:c r="R107" s="72"/>
+      <x:c r="S107" s="72"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="21"/>
@@ -2871,6 +3318,10 @@
       <x:c r="M108" s="26"/>
       <x:c r="N108" s="26"/>
       <x:c r="O108" s="27"/>
+      <x:c r="P108" s="72"/>
+      <x:c r="Q108" s="72"/>
+      <x:c r="R108" s="72"/>
+      <x:c r="S108" s="72"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="21"/>
@@ -2888,6 +3339,10 @@
       <x:c r="M109" s="26"/>
       <x:c r="N109" s="26"/>
       <x:c r="O109" s="27"/>
+      <x:c r="P109" s="72"/>
+      <x:c r="Q109" s="72"/>
+      <x:c r="R109" s="72"/>
+      <x:c r="S109" s="72"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="21"/>
@@ -2905,6 +3360,10 @@
       <x:c r="M110" s="26"/>
       <x:c r="N110" s="26"/>
       <x:c r="O110" s="27"/>
+      <x:c r="P110" s="72"/>
+      <x:c r="Q110" s="72"/>
+      <x:c r="R110" s="72"/>
+      <x:c r="S110" s="72"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="21"/>
@@ -2922,6 +3381,10 @@
       <x:c r="M111" s="26"/>
       <x:c r="N111" s="26"/>
       <x:c r="O111" s="27"/>
+      <x:c r="P111" s="72"/>
+      <x:c r="Q111" s="72"/>
+      <x:c r="R111" s="72"/>
+      <x:c r="S111" s="72"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="21"/>
@@ -2939,6 +3402,10 @@
       <x:c r="M112" s="26"/>
       <x:c r="N112" s="26"/>
       <x:c r="O112" s="27"/>
+      <x:c r="P112" s="72"/>
+      <x:c r="Q112" s="72"/>
+      <x:c r="R112" s="72"/>
+      <x:c r="S112" s="72"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="21"/>
@@ -2956,6 +3423,10 @@
       <x:c r="M113" s="26"/>
       <x:c r="N113" s="26"/>
       <x:c r="O113" s="27"/>
+      <x:c r="P113" s="72"/>
+      <x:c r="Q113" s="72"/>
+      <x:c r="R113" s="72"/>
+      <x:c r="S113" s="72"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="21"/>
@@ -2973,6 +3444,10 @@
       <x:c r="M114" s="26"/>
       <x:c r="N114" s="26"/>
       <x:c r="O114" s="27"/>
+      <x:c r="P114" s="72"/>
+      <x:c r="Q114" s="72"/>
+      <x:c r="R114" s="72"/>
+      <x:c r="S114" s="72"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="21"/>
@@ -2990,6 +3465,10 @@
       <x:c r="M115" s="26"/>
       <x:c r="N115" s="26"/>
       <x:c r="O115" s="27"/>
+      <x:c r="P115" s="72"/>
+      <x:c r="Q115" s="72"/>
+      <x:c r="R115" s="72"/>
+      <x:c r="S115" s="72"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="21"/>
@@ -3007,6 +3486,10 @@
       <x:c r="M116" s="26"/>
       <x:c r="N116" s="26"/>
       <x:c r="O116" s="27"/>
+      <x:c r="P116" s="72"/>
+      <x:c r="Q116" s="72"/>
+      <x:c r="R116" s="72"/>
+      <x:c r="S116" s="72"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="21"/>
@@ -3024,6 +3507,10 @@
       <x:c r="M117" s="26"/>
       <x:c r="N117" s="26"/>
       <x:c r="O117" s="27"/>
+      <x:c r="P117" s="72"/>
+      <x:c r="Q117" s="72"/>
+      <x:c r="R117" s="72"/>
+      <x:c r="S117" s="72"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="21"/>
@@ -3041,6 +3528,10 @@
       <x:c r="M118" s="26"/>
       <x:c r="N118" s="26"/>
       <x:c r="O118" s="27"/>
+      <x:c r="P118" s="72"/>
+      <x:c r="Q118" s="72"/>
+      <x:c r="R118" s="72"/>
+      <x:c r="S118" s="72"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="21"/>
@@ -3058,6 +3549,10 @@
       <x:c r="M119" s="26"/>
       <x:c r="N119" s="26"/>
       <x:c r="O119" s="27"/>
+      <x:c r="P119" s="72"/>
+      <x:c r="Q119" s="72"/>
+      <x:c r="R119" s="72"/>
+      <x:c r="S119" s="72"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="21"/>
@@ -3075,6 +3570,10 @@
       <x:c r="M120" s="26"/>
       <x:c r="N120" s="26"/>
       <x:c r="O120" s="27"/>
+      <x:c r="P120" s="72"/>
+      <x:c r="Q120" s="72"/>
+      <x:c r="R120" s="72"/>
+      <x:c r="S120" s="72"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="21"/>
@@ -3092,6 +3591,10 @@
       <x:c r="M121" s="26"/>
       <x:c r="N121" s="26"/>
       <x:c r="O121" s="27"/>
+      <x:c r="P121" s="72"/>
+      <x:c r="Q121" s="72"/>
+      <x:c r="R121" s="72"/>
+      <x:c r="S121" s="72"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="21"/>
@@ -3109,6 +3612,10 @@
       <x:c r="M122" s="26"/>
       <x:c r="N122" s="26"/>
       <x:c r="O122" s="27"/>
+      <x:c r="P122" s="72"/>
+      <x:c r="Q122" s="72"/>
+      <x:c r="R122" s="72"/>
+      <x:c r="S122" s="72"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="21"/>
@@ -3126,6 +3633,10 @@
       <x:c r="M123" s="26"/>
       <x:c r="N123" s="26"/>
       <x:c r="O123" s="27"/>
+      <x:c r="P123" s="72"/>
+      <x:c r="Q123" s="72"/>
+      <x:c r="R123" s="72"/>
+      <x:c r="S123" s="72"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="21"/>
@@ -3143,6 +3654,10 @@
       <x:c r="M124" s="26"/>
       <x:c r="N124" s="26"/>
       <x:c r="O124" s="27"/>
+      <x:c r="P124" s="72"/>
+      <x:c r="Q124" s="72"/>
+      <x:c r="R124" s="72"/>
+      <x:c r="S124" s="72"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="21"/>
@@ -3160,6 +3675,10 @@
       <x:c r="M125" s="26"/>
       <x:c r="N125" s="26"/>
       <x:c r="O125" s="27"/>
+      <x:c r="P125" s="72"/>
+      <x:c r="Q125" s="72"/>
+      <x:c r="R125" s="72"/>
+      <x:c r="S125" s="72"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="21"/>
@@ -3177,6 +3696,10 @@
       <x:c r="M126" s="26"/>
       <x:c r="N126" s="26"/>
       <x:c r="O126" s="27"/>
+      <x:c r="P126" s="72"/>
+      <x:c r="Q126" s="72"/>
+      <x:c r="R126" s="72"/>
+      <x:c r="S126" s="72"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="21"/>
@@ -3194,6 +3717,10 @@
       <x:c r="M127" s="26"/>
       <x:c r="N127" s="26"/>
       <x:c r="O127" s="27"/>
+      <x:c r="P127" s="72"/>
+      <x:c r="Q127" s="72"/>
+      <x:c r="R127" s="72"/>
+      <x:c r="S127" s="72"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="21"/>
@@ -3211,6 +3738,10 @@
       <x:c r="M128" s="26"/>
       <x:c r="N128" s="26"/>
       <x:c r="O128" s="27"/>
+      <x:c r="P128" s="72"/>
+      <x:c r="Q128" s="72"/>
+      <x:c r="R128" s="72"/>
+      <x:c r="S128" s="72"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="21"/>
@@ -3228,6 +3759,10 @@
       <x:c r="M129" s="26"/>
       <x:c r="N129" s="26"/>
       <x:c r="O129" s="27"/>
+      <x:c r="P129" s="72"/>
+      <x:c r="Q129" s="72"/>
+      <x:c r="R129" s="72"/>
+      <x:c r="S129" s="72"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="21"/>
@@ -3245,6 +3780,10 @@
       <x:c r="M130" s="26"/>
       <x:c r="N130" s="26"/>
       <x:c r="O130" s="27"/>
+      <x:c r="P130" s="72"/>
+      <x:c r="Q130" s="72"/>
+      <x:c r="R130" s="72"/>
+      <x:c r="S130" s="72"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="21"/>
@@ -3262,6 +3801,10 @@
       <x:c r="M131" s="26"/>
       <x:c r="N131" s="26"/>
       <x:c r="O131" s="27"/>
+      <x:c r="P131" s="72"/>
+      <x:c r="Q131" s="72"/>
+      <x:c r="R131" s="72"/>
+      <x:c r="S131" s="72"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="21"/>
@@ -3279,6 +3822,10 @@
       <x:c r="M132" s="26"/>
       <x:c r="N132" s="26"/>
       <x:c r="O132" s="27"/>
+      <x:c r="P132" s="72"/>
+      <x:c r="Q132" s="72"/>
+      <x:c r="R132" s="72"/>
+      <x:c r="S132" s="72"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="21"/>
@@ -3296,6 +3843,10 @@
       <x:c r="M133" s="26"/>
       <x:c r="N133" s="26"/>
       <x:c r="O133" s="27"/>
+      <x:c r="P133" s="72"/>
+      <x:c r="Q133" s="72"/>
+      <x:c r="R133" s="72"/>
+      <x:c r="S133" s="72"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="21"/>
@@ -3313,6 +3864,10 @@
       <x:c r="M134" s="26"/>
       <x:c r="N134" s="26"/>
       <x:c r="O134" s="27"/>
+      <x:c r="P134" s="72"/>
+      <x:c r="Q134" s="72"/>
+      <x:c r="R134" s="72"/>
+      <x:c r="S134" s="72"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="21"/>
@@ -3330,6 +3885,10 @@
       <x:c r="M135" s="26"/>
       <x:c r="N135" s="26"/>
       <x:c r="O135" s="27"/>
+      <x:c r="P135" s="72"/>
+      <x:c r="Q135" s="72"/>
+      <x:c r="R135" s="72"/>
+      <x:c r="S135" s="72"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="21"/>
@@ -3347,6 +3906,10 @@
       <x:c r="M136" s="26"/>
       <x:c r="N136" s="26"/>
       <x:c r="O136" s="27"/>
+      <x:c r="P136" s="72"/>
+      <x:c r="Q136" s="72"/>
+      <x:c r="R136" s="72"/>
+      <x:c r="S136" s="72"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="21"/>
@@ -3364,6 +3927,10 @@
       <x:c r="M137" s="26"/>
       <x:c r="N137" s="26"/>
       <x:c r="O137" s="27"/>
+      <x:c r="P137" s="72"/>
+      <x:c r="Q137" s="72"/>
+      <x:c r="R137" s="72"/>
+      <x:c r="S137" s="72"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="21"/>
@@ -3381,6 +3948,10 @@
       <x:c r="M138" s="26"/>
       <x:c r="N138" s="26"/>
       <x:c r="O138" s="27"/>
+      <x:c r="P138" s="72"/>
+      <x:c r="Q138" s="72"/>
+      <x:c r="R138" s="72"/>
+      <x:c r="S138" s="72"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="21"/>
@@ -3398,6 +3969,10 @@
       <x:c r="M139" s="26"/>
       <x:c r="N139" s="26"/>
       <x:c r="O139" s="27"/>
+      <x:c r="P139" s="72"/>
+      <x:c r="Q139" s="72"/>
+      <x:c r="R139" s="72"/>
+      <x:c r="S139" s="72"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="21"/>
@@ -3415,6 +3990,10 @@
       <x:c r="M140" s="26"/>
       <x:c r="N140" s="26"/>
       <x:c r="O140" s="27"/>
+      <x:c r="P140" s="72"/>
+      <x:c r="Q140" s="72"/>
+      <x:c r="R140" s="72"/>
+      <x:c r="S140" s="72"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="21"/>
@@ -3432,6 +4011,10 @@
       <x:c r="M141" s="26"/>
       <x:c r="N141" s="26"/>
       <x:c r="O141" s="27"/>
+      <x:c r="P141" s="72"/>
+      <x:c r="Q141" s="72"/>
+      <x:c r="R141" s="72"/>
+      <x:c r="S141" s="72"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="21"/>
@@ -3449,6 +4032,10 @@
       <x:c r="M142" s="26"/>
       <x:c r="N142" s="26"/>
       <x:c r="O142" s="27"/>
+      <x:c r="P142" s="72"/>
+      <x:c r="Q142" s="72"/>
+      <x:c r="R142" s="72"/>
+      <x:c r="S142" s="72"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="21"/>
@@ -3466,6 +4053,10 @@
       <x:c r="M143" s="26"/>
       <x:c r="N143" s="26"/>
       <x:c r="O143" s="27"/>
+      <x:c r="P143" s="72"/>
+      <x:c r="Q143" s="72"/>
+      <x:c r="R143" s="72"/>
+      <x:c r="S143" s="72"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="21"/>
@@ -3483,6 +4074,10 @@
       <x:c r="M144" s="26"/>
       <x:c r="N144" s="26"/>
       <x:c r="O144" s="27"/>
+      <x:c r="P144" s="72"/>
+      <x:c r="Q144" s="72"/>
+      <x:c r="R144" s="72"/>
+      <x:c r="S144" s="72"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="21"/>
@@ -3500,6 +4095,10 @@
       <x:c r="M145" s="26"/>
       <x:c r="N145" s="26"/>
       <x:c r="O145" s="27"/>
+      <x:c r="P145" s="72"/>
+      <x:c r="Q145" s="72"/>
+      <x:c r="R145" s="72"/>
+      <x:c r="S145" s="72"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="21"/>
@@ -3517,6 +4116,10 @@
       <x:c r="M146" s="26"/>
       <x:c r="N146" s="26"/>
       <x:c r="O146" s="27"/>
+      <x:c r="P146" s="72"/>
+      <x:c r="Q146" s="72"/>
+      <x:c r="R146" s="72"/>
+      <x:c r="S146" s="72"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="21"/>
@@ -3534,6 +4137,10 @@
       <x:c r="M147" s="26"/>
       <x:c r="N147" s="26"/>
       <x:c r="O147" s="27"/>
+      <x:c r="P147" s="72"/>
+      <x:c r="Q147" s="72"/>
+      <x:c r="R147" s="72"/>
+      <x:c r="S147" s="72"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="21"/>
@@ -3551,6 +4158,10 @@
       <x:c r="M148" s="26"/>
       <x:c r="N148" s="26"/>
       <x:c r="O148" s="27"/>
+      <x:c r="P148" s="72"/>
+      <x:c r="Q148" s="72"/>
+      <x:c r="R148" s="72"/>
+      <x:c r="S148" s="72"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="21"/>
@@ -3568,6 +4179,10 @@
       <x:c r="M149" s="26"/>
       <x:c r="N149" s="26"/>
       <x:c r="O149" s="27"/>
+      <x:c r="P149" s="72"/>
+      <x:c r="Q149" s="72"/>
+      <x:c r="R149" s="72"/>
+      <x:c r="S149" s="72"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="21"/>
@@ -3585,6 +4200,10 @@
       <x:c r="M150" s="26"/>
       <x:c r="N150" s="26"/>
       <x:c r="O150" s="27"/>
+      <x:c r="P150" s="72"/>
+      <x:c r="Q150" s="72"/>
+      <x:c r="R150" s="72"/>
+      <x:c r="S150" s="72"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="21"/>
@@ -3602,6 +4221,10 @@
       <x:c r="M151" s="26"/>
       <x:c r="N151" s="26"/>
       <x:c r="O151" s="27"/>
+      <x:c r="P151" s="72"/>
+      <x:c r="Q151" s="72"/>
+      <x:c r="R151" s="72"/>
+      <x:c r="S151" s="72"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="21"/>
@@ -3619,6 +4242,10 @@
       <x:c r="M152" s="26"/>
       <x:c r="N152" s="26"/>
       <x:c r="O152" s="27"/>
+      <x:c r="P152" s="72"/>
+      <x:c r="Q152" s="72"/>
+      <x:c r="R152" s="72"/>
+      <x:c r="S152" s="72"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="21"/>
@@ -3636,6 +4263,10 @@
       <x:c r="M153" s="26"/>
       <x:c r="N153" s="26"/>
       <x:c r="O153" s="27"/>
+      <x:c r="P153" s="72"/>
+      <x:c r="Q153" s="72"/>
+      <x:c r="R153" s="72"/>
+      <x:c r="S153" s="72"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="21"/>
@@ -3653,6 +4284,10 @@
       <x:c r="M154" s="26"/>
       <x:c r="N154" s="26"/>
       <x:c r="O154" s="27"/>
+      <x:c r="P154" s="72"/>
+      <x:c r="Q154" s="72"/>
+      <x:c r="R154" s="72"/>
+      <x:c r="S154" s="72"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="21"/>
@@ -3670,6 +4305,10 @@
       <x:c r="M155" s="26"/>
       <x:c r="N155" s="26"/>
       <x:c r="O155" s="27"/>
+      <x:c r="P155" s="72"/>
+      <x:c r="Q155" s="72"/>
+      <x:c r="R155" s="72"/>
+      <x:c r="S155" s="72"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="21"/>
@@ -3687,6 +4326,10 @@
       <x:c r="M156" s="26"/>
       <x:c r="N156" s="26"/>
       <x:c r="O156" s="27"/>
+      <x:c r="P156" s="72"/>
+      <x:c r="Q156" s="72"/>
+      <x:c r="R156" s="72"/>
+      <x:c r="S156" s="72"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="21"/>
@@ -3704,6 +4347,10 @@
       <x:c r="M157" s="26"/>
       <x:c r="N157" s="26"/>
       <x:c r="O157" s="27"/>
+      <x:c r="P157" s="72"/>
+      <x:c r="Q157" s="72"/>
+      <x:c r="R157" s="72"/>
+      <x:c r="S157" s="72"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="21"/>
@@ -3721,6 +4368,10 @@
       <x:c r="M158" s="26"/>
       <x:c r="N158" s="26"/>
       <x:c r="O158" s="27"/>
+      <x:c r="P158" s="72"/>
+      <x:c r="Q158" s="72"/>
+      <x:c r="R158" s="72"/>
+      <x:c r="S158" s="72"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="21"/>
@@ -3738,6 +4389,10 @@
       <x:c r="M159" s="26"/>
       <x:c r="N159" s="26"/>
       <x:c r="O159" s="27"/>
+      <x:c r="P159" s="72"/>
+      <x:c r="Q159" s="72"/>
+      <x:c r="R159" s="72"/>
+      <x:c r="S159" s="72"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="21"/>
@@ -3755,6 +4410,10 @@
       <x:c r="M160" s="26"/>
       <x:c r="N160" s="26"/>
       <x:c r="O160" s="27"/>
+      <x:c r="P160" s="72"/>
+      <x:c r="Q160" s="72"/>
+      <x:c r="R160" s="72"/>
+      <x:c r="S160" s="72"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="21"/>
@@ -3772,6 +4431,10 @@
       <x:c r="M161" s="26"/>
       <x:c r="N161" s="26"/>
       <x:c r="O161" s="27"/>
+      <x:c r="P161" s="72"/>
+      <x:c r="Q161" s="72"/>
+      <x:c r="R161" s="72"/>
+      <x:c r="S161" s="72"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="21"/>
@@ -3789,6 +4452,10 @@
       <x:c r="M162" s="26"/>
       <x:c r="N162" s="26"/>
       <x:c r="O162" s="27"/>
+      <x:c r="P162" s="72"/>
+      <x:c r="Q162" s="72"/>
+      <x:c r="R162" s="72"/>
+      <x:c r="S162" s="72"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="21"/>
@@ -3806,6 +4473,10 @@
       <x:c r="M163" s="26"/>
       <x:c r="N163" s="26"/>
       <x:c r="O163" s="27"/>
+      <x:c r="P163" s="72"/>
+      <x:c r="Q163" s="72"/>
+      <x:c r="R163" s="72"/>
+      <x:c r="S163" s="72"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="21"/>
@@ -3823,6 +4494,10 @@
       <x:c r="M164" s="26"/>
       <x:c r="N164" s="26"/>
       <x:c r="O164" s="27"/>
+      <x:c r="P164" s="72"/>
+      <x:c r="Q164" s="72"/>
+      <x:c r="R164" s="72"/>
+      <x:c r="S164" s="72"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="21"/>
@@ -3840,6 +4515,10 @@
       <x:c r="M165" s="26"/>
       <x:c r="N165" s="26"/>
       <x:c r="O165" s="27"/>
+      <x:c r="P165" s="72"/>
+      <x:c r="Q165" s="72"/>
+      <x:c r="R165" s="72"/>
+      <x:c r="S165" s="72"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="21"/>
@@ -3857,6 +4536,10 @@
       <x:c r="M166" s="26"/>
       <x:c r="N166" s="26"/>
       <x:c r="O166" s="27"/>
+      <x:c r="P166" s="72"/>
+      <x:c r="Q166" s="72"/>
+      <x:c r="R166" s="72"/>
+      <x:c r="S166" s="72"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="21"/>
@@ -3874,6 +4557,10 @@
       <x:c r="M167" s="26"/>
       <x:c r="N167" s="26"/>
       <x:c r="O167" s="27"/>
+      <x:c r="P167" s="72"/>
+      <x:c r="Q167" s="72"/>
+      <x:c r="R167" s="72"/>
+      <x:c r="S167" s="72"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="21"/>
@@ -3891,6 +4578,10 @@
       <x:c r="M168" s="26"/>
       <x:c r="N168" s="26"/>
       <x:c r="O168" s="27"/>
+      <x:c r="P168" s="72"/>
+      <x:c r="Q168" s="72"/>
+      <x:c r="R168" s="72"/>
+      <x:c r="S168" s="72"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="21"/>
@@ -3908,6 +4599,10 @@
       <x:c r="M169" s="26"/>
       <x:c r="N169" s="26"/>
       <x:c r="O169" s="27"/>
+      <x:c r="P169" s="72"/>
+      <x:c r="Q169" s="72"/>
+      <x:c r="R169" s="72"/>
+      <x:c r="S169" s="72"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="21"/>
@@ -3925,6 +4620,10 @@
       <x:c r="M170" s="26"/>
       <x:c r="N170" s="26"/>
       <x:c r="O170" s="27"/>
+      <x:c r="P170" s="72"/>
+      <x:c r="Q170" s="72"/>
+      <x:c r="R170" s="72"/>
+      <x:c r="S170" s="72"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="21"/>
@@ -3942,6 +4641,10 @@
       <x:c r="M171" s="26"/>
       <x:c r="N171" s="26"/>
       <x:c r="O171" s="27"/>
+      <x:c r="P171" s="72"/>
+      <x:c r="Q171" s="72"/>
+      <x:c r="R171" s="72"/>
+      <x:c r="S171" s="72"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="21"/>
@@ -3959,6 +4662,10 @@
       <x:c r="M172" s="26"/>
       <x:c r="N172" s="26"/>
       <x:c r="O172" s="27"/>
+      <x:c r="P172" s="72"/>
+      <x:c r="Q172" s="72"/>
+      <x:c r="R172" s="72"/>
+      <x:c r="S172" s="72"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="21"/>
@@ -3976,6 +4683,10 @@
       <x:c r="M173" s="26"/>
       <x:c r="N173" s="26"/>
       <x:c r="O173" s="27"/>
+      <x:c r="P173" s="72"/>
+      <x:c r="Q173" s="72"/>
+      <x:c r="R173" s="72"/>
+      <x:c r="S173" s="72"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="21"/>
@@ -3993,6 +4704,10 @@
       <x:c r="M174" s="26"/>
       <x:c r="N174" s="26"/>
       <x:c r="O174" s="27"/>
+      <x:c r="P174" s="72"/>
+      <x:c r="Q174" s="72"/>
+      <x:c r="R174" s="72"/>
+      <x:c r="S174" s="72"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="21"/>
@@ -4010,6 +4725,10 @@
       <x:c r="M175" s="26"/>
       <x:c r="N175" s="26"/>
       <x:c r="O175" s="27"/>
+      <x:c r="P175" s="72"/>
+      <x:c r="Q175" s="72"/>
+      <x:c r="R175" s="72"/>
+      <x:c r="S175" s="72"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="21"/>
@@ -4027,6 +4746,10 @@
       <x:c r="M176" s="26"/>
       <x:c r="N176" s="26"/>
       <x:c r="O176" s="27"/>
+      <x:c r="P176" s="72"/>
+      <x:c r="Q176" s="72"/>
+      <x:c r="R176" s="72"/>
+      <x:c r="S176" s="72"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="21"/>
@@ -4044,6 +4767,10 @@
       <x:c r="M177" s="26"/>
       <x:c r="N177" s="26"/>
       <x:c r="O177" s="27"/>
+      <x:c r="P177" s="72"/>
+      <x:c r="Q177" s="72"/>
+      <x:c r="R177" s="72"/>
+      <x:c r="S177" s="72"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="21"/>
@@ -4061,6 +4788,10 @@
       <x:c r="M178" s="26"/>
       <x:c r="N178" s="26"/>
       <x:c r="O178" s="27"/>
+      <x:c r="P178" s="72"/>
+      <x:c r="Q178" s="72"/>
+      <x:c r="R178" s="72"/>
+      <x:c r="S178" s="72"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="21"/>
@@ -4078,6 +4809,10 @@
       <x:c r="M179" s="26"/>
       <x:c r="N179" s="26"/>
       <x:c r="O179" s="27"/>
+      <x:c r="P179" s="72"/>
+      <x:c r="Q179" s="72"/>
+      <x:c r="R179" s="72"/>
+      <x:c r="S179" s="72"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="21"/>
@@ -4095,6 +4830,10 @@
       <x:c r="M180" s="26"/>
       <x:c r="N180" s="26"/>
       <x:c r="O180" s="27"/>
+      <x:c r="P180" s="72"/>
+      <x:c r="Q180" s="72"/>
+      <x:c r="R180" s="72"/>
+      <x:c r="S180" s="72"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="21"/>
@@ -4112,6 +4851,10 @@
       <x:c r="M181" s="26"/>
       <x:c r="N181" s="26"/>
       <x:c r="O181" s="27"/>
+      <x:c r="P181" s="72"/>
+      <x:c r="Q181" s="72"/>
+      <x:c r="R181" s="72"/>
+      <x:c r="S181" s="72"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="21"/>
@@ -4129,6 +4872,10 @@
       <x:c r="M182" s="26"/>
       <x:c r="N182" s="26"/>
       <x:c r="O182" s="27"/>
+      <x:c r="P182" s="72"/>
+      <x:c r="Q182" s="72"/>
+      <x:c r="R182" s="72"/>
+      <x:c r="S182" s="72"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="21"/>
@@ -4146,6 +4893,10 @@
       <x:c r="M183" s="26"/>
       <x:c r="N183" s="26"/>
       <x:c r="O183" s="27"/>
+      <x:c r="P183" s="72"/>
+      <x:c r="Q183" s="72"/>
+      <x:c r="R183" s="72"/>
+      <x:c r="S183" s="72"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="21"/>
@@ -4163,6 +4914,10 @@
       <x:c r="M184" s="26"/>
       <x:c r="N184" s="26"/>
       <x:c r="O184" s="27"/>
+      <x:c r="P184" s="72"/>
+      <x:c r="Q184" s="72"/>
+      <x:c r="R184" s="72"/>
+      <x:c r="S184" s="72"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="21"/>
@@ -4180,6 +4935,10 @@
       <x:c r="M185" s="26"/>
       <x:c r="N185" s="26"/>
       <x:c r="O185" s="27"/>
+      <x:c r="P185" s="72"/>
+      <x:c r="Q185" s="72"/>
+      <x:c r="R185" s="72"/>
+      <x:c r="S185" s="72"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="21"/>
@@ -4197,6 +4956,10 @@
       <x:c r="M186" s="26"/>
       <x:c r="N186" s="26"/>
       <x:c r="O186" s="27"/>
+      <x:c r="P186" s="72"/>
+      <x:c r="Q186" s="72"/>
+      <x:c r="R186" s="72"/>
+      <x:c r="S186" s="72"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="21"/>
@@ -4214,6 +4977,10 @@
       <x:c r="M187" s="26"/>
       <x:c r="N187" s="26"/>
       <x:c r="O187" s="27"/>
+      <x:c r="P187" s="72"/>
+      <x:c r="Q187" s="72"/>
+      <x:c r="R187" s="72"/>
+      <x:c r="S187" s="72"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="21"/>
@@ -4231,6 +4998,10 @@
       <x:c r="M188" s="26"/>
       <x:c r="N188" s="26"/>
       <x:c r="O188" s="27"/>
+      <x:c r="P188" s="72"/>
+      <x:c r="Q188" s="72"/>
+      <x:c r="R188" s="72"/>
+      <x:c r="S188" s="72"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="21"/>
@@ -4248,6 +5019,10 @@
       <x:c r="M189" s="26"/>
       <x:c r="N189" s="26"/>
       <x:c r="O189" s="27"/>
+      <x:c r="P189" s="72"/>
+      <x:c r="Q189" s="72"/>
+      <x:c r="R189" s="72"/>
+      <x:c r="S189" s="72"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="21"/>
@@ -4265,6 +5040,10 @@
       <x:c r="M190" s="26"/>
       <x:c r="N190" s="26"/>
       <x:c r="O190" s="27"/>
+      <x:c r="P190" s="72"/>
+      <x:c r="Q190" s="72"/>
+      <x:c r="R190" s="72"/>
+      <x:c r="S190" s="72"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="21"/>
@@ -4282,6 +5061,10 @@
       <x:c r="M191" s="26"/>
       <x:c r="N191" s="26"/>
       <x:c r="O191" s="27"/>
+      <x:c r="P191" s="72"/>
+      <x:c r="Q191" s="72"/>
+      <x:c r="R191" s="72"/>
+      <x:c r="S191" s="72"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="21"/>
@@ -4299,6 +5082,10 @@
       <x:c r="M192" s="26"/>
       <x:c r="N192" s="26"/>
       <x:c r="O192" s="27"/>
+      <x:c r="P192" s="72"/>
+      <x:c r="Q192" s="72"/>
+      <x:c r="R192" s="72"/>
+      <x:c r="S192" s="72"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="21"/>
@@ -4316,6 +5103,10 @@
       <x:c r="M193" s="26"/>
       <x:c r="N193" s="26"/>
       <x:c r="O193" s="27"/>
+      <x:c r="P193" s="72"/>
+      <x:c r="Q193" s="72"/>
+      <x:c r="R193" s="72"/>
+      <x:c r="S193" s="72"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="21"/>
@@ -4333,6 +5124,10 @@
       <x:c r="M194" s="26"/>
       <x:c r="N194" s="26"/>
       <x:c r="O194" s="27"/>
+      <x:c r="P194" s="72"/>
+      <x:c r="Q194" s="72"/>
+      <x:c r="R194" s="72"/>
+      <x:c r="S194" s="72"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="21"/>
@@ -4350,6 +5145,10 @@
       <x:c r="M195" s="26"/>
       <x:c r="N195" s="26"/>
       <x:c r="O195" s="27"/>
+      <x:c r="P195" s="72"/>
+      <x:c r="Q195" s="72"/>
+      <x:c r="R195" s="72"/>
+      <x:c r="S195" s="72"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="21"/>
@@ -4367,6 +5166,10 @@
       <x:c r="M196" s="26"/>
       <x:c r="N196" s="26"/>
       <x:c r="O196" s="27"/>
+      <x:c r="P196" s="72"/>
+      <x:c r="Q196" s="72"/>
+      <x:c r="R196" s="72"/>
+      <x:c r="S196" s="72"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="21"/>
@@ -4384,6 +5187,10 @@
       <x:c r="M197" s="26"/>
       <x:c r="N197" s="26"/>
       <x:c r="O197" s="27"/>
+      <x:c r="P197" s="72"/>
+      <x:c r="Q197" s="72"/>
+      <x:c r="R197" s="72"/>
+      <x:c r="S197" s="72"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="21"/>
@@ -4401,6 +5208,10 @@
       <x:c r="M198" s="26"/>
       <x:c r="N198" s="26"/>
       <x:c r="O198" s="27"/>
+      <x:c r="P198" s="72"/>
+      <x:c r="Q198" s="72"/>
+      <x:c r="R198" s="72"/>
+      <x:c r="S198" s="72"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="21"/>
@@ -4418,6 +5229,10 @@
       <x:c r="M199" s="26"/>
       <x:c r="N199" s="26"/>
       <x:c r="O199" s="27"/>
+      <x:c r="P199" s="72"/>
+      <x:c r="Q199" s="72"/>
+      <x:c r="R199" s="72"/>
+      <x:c r="S199" s="72"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="21"/>
@@ -4435,6 +5250,10 @@
       <x:c r="M200" s="26"/>
       <x:c r="N200" s="26"/>
       <x:c r="O200" s="27"/>
+      <x:c r="P200" s="72"/>
+      <x:c r="Q200" s="72"/>
+      <x:c r="R200" s="72"/>
+      <x:c r="S200" s="72"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="21"/>
@@ -4452,6 +5271,10 @@
       <x:c r="M201" s="26"/>
       <x:c r="N201" s="26"/>
       <x:c r="O201" s="27"/>
+      <x:c r="P201" s="72"/>
+      <x:c r="Q201" s="72"/>
+      <x:c r="R201" s="72"/>
+      <x:c r="S201" s="72"/>
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="21"/>
@@ -4469,6 +5292,10 @@
       <x:c r="M202" s="26"/>
       <x:c r="N202" s="26"/>
       <x:c r="O202" s="27"/>
+      <x:c r="P202" s="72"/>
+      <x:c r="Q202" s="72"/>
+      <x:c r="R202" s="72"/>
+      <x:c r="S202" s="72"/>
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="30"/>
@@ -4486,6 +5313,10 @@
       <x:c r="M203" s="28"/>
       <x:c r="N203" s="28"/>
       <x:c r="O203" s="29"/>
+      <x:c r="P203" s="72"/>
+      <x:c r="Q203" s="72"/>
+      <x:c r="R203" s="72"/>
+      <x:c r="S203" s="72"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4499,7 +5330,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1b0613789a04602"/>
+    <x:tablePart ns1:id="Rf1b0613789a04602"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>